<commit_message>
Updated Disk, Grub, Git & KVM
</commit_message>
<xml_diff>
--- a/disks-partitioning.xlsx
+++ b/disks-partitioning.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t xml:space="preserve">80 GiB VM</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">VFAT(fat32) /EFI</t>
   </si>
   <si>
-    <t xml:space="preserve">1024 MiB</t>
+    <t xml:space="preserve">600 MiB (7.1M-41M)</t>
   </si>
   <si>
     <t xml:space="preserve">/boot</t>
@@ -58,10 +58,13 @@
     <t xml:space="preserve">ext2,ext4,xfs</t>
   </si>
   <si>
+    <t xml:space="preserve">1024 MiB (226M-814M)</t>
+  </si>
+  <si>
     <t xml:space="preserve">/</t>
   </si>
   <si>
-    <t xml:space="preserve">etx4,XFS</t>
+    <t xml:space="preserve">ext4,XFS</t>
   </si>
   <si>
     <t xml:space="preserve">20 to LARGE</t>
@@ -582,10 +585,10 @@
         <v>0.6</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>2</v>
+        <v>0.6</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -596,7 +599,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>1</v>
@@ -605,21 +608,21 @@
         <v>1</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>2.4</v>
@@ -636,13 +639,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>2</v>
@@ -659,13 +662,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>3</v>
@@ -682,13 +685,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>3</v>
@@ -705,13 +708,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -728,13 +731,13 @@
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>4</v>
@@ -751,10 +754,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>2</v>
@@ -771,13 +774,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0</v>
@@ -788,13 +791,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -805,13 +808,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
@@ -822,7 +825,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D17" s="1" t="n">
         <f aca="false">SUM(D2:D15)</f>
@@ -834,7 +837,7 @@
       </c>
       <c r="F17" s="1" t="n">
         <f aca="false">SUM(F2:F16)</f>
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="G17" s="1" t="n">
         <f aca="false">SUM(G2:G16)</f>
@@ -843,154 +846,154 @@
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Update Grub & Disks Partitioning
</commit_message>
<xml_diff>
--- a/disks-partitioning.xlsx
+++ b/disks-partitioning.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">VFAT / EFI / ESP</t>
   </si>
   <si>
-    <t xml:space="preserve">600 MiB (7.1M-41M)</t>
+    <t xml:space="preserve">600 MiB (7.1M-41M) (PRESERVE)</t>
   </si>
   <si>
     <t xml:space="preserve">/boot</t>
@@ -100,7 +100,8 @@
     <t xml:space="preserve">[SWAP]</t>
   </si>
   <si>
-    <t xml:space="preserve">ZRAM optional</t>
+    <t xml:space="preserve">ZRAM optional
+(PRESERVE SWAP FOR USE ON ALL OS’S)</t>
   </si>
   <si>
     <t xml:space="preserve">4 for 16Gb RAM
@@ -441,9 +442,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>717480</xdr:colOff>
+      <xdr:colOff>716760</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>152640</xdr:rowOff>
+      <xdr:rowOff>151920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -456,8 +457,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6424560" y="2531880"/>
-          <a:ext cx="4360320" cy="3216240"/>
+          <a:off x="6423840" y="2531880"/>
+          <a:ext cx="4359600" cy="3215520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -784,7 +785,7 @@
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C10" s="2" t="s">

</xml_diff>

<commit_message>
Update Grub and Disk Partitions file
</commit_message>
<xml_diff>
--- a/disks-partitioning.xlsx
+++ b/disks-partitioning.xlsx
@@ -282,12 +282,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -330,7 +336,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -344,6 +350,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -412,7 +422,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -442,9 +452,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>716760</xdr:colOff>
+      <xdr:colOff>716400</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>151920</xdr:rowOff>
+      <xdr:rowOff>151560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -458,7 +468,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6423840" y="2531880"/>
-          <a:ext cx="4359600" cy="3215520"/>
+          <a:ext cx="4359240" cy="3215160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -616,7 +626,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -667,7 +677,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -782,7 +792,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -825,58 +835,58 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>34</v>
       </c>
       <c r="D17" s="1" t="n">
@@ -897,10 +907,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>36</v>
       </c>
     </row>
@@ -908,7 +918,7 @@
       <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -916,7 +926,7 @@
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>40</v>
       </c>
     </row>
@@ -924,7 +934,7 @@
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>42</v>
       </c>
     </row>
@@ -932,7 +942,7 @@
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>44</v>
       </c>
     </row>
@@ -940,7 +950,7 @@
       <c r="A23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>46</v>
       </c>
     </row>
@@ -948,7 +958,7 @@
       <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>48</v>
       </c>
     </row>
@@ -956,7 +966,7 @@
       <c r="A25" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>50</v>
       </c>
     </row>
@@ -964,7 +974,7 @@
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>52</v>
       </c>
     </row>
@@ -972,7 +982,7 @@
       <c r="A27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -980,7 +990,7 @@
       <c r="A28" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>56</v>
       </c>
     </row>
@@ -988,7 +998,7 @@
       <c r="A29" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>58</v>
       </c>
     </row>
@@ -996,7 +1006,7 @@
       <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1004,7 +1014,7 @@
       <c r="A31" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1012,7 +1022,7 @@
       <c r="A32" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1020,7 +1030,7 @@
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1028,7 +1038,7 @@
       <c r="A34" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1036,7 +1046,7 @@
       <c r="A35" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1044,7 +1054,7 @@
       <c r="A36" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Disks Partitioning for MX
</commit_message>
<xml_diff>
--- a/disks-partitioning.xlsx
+++ b/disks-partitioning.xlsx
@@ -452,9 +452,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>716400</xdr:colOff>
+      <xdr:colOff>716040</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>151560</xdr:rowOff>
+      <xdr:rowOff>151200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -468,7 +468,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6423840" y="2531880"/>
-          <a:ext cx="4359240" cy="3215160"/>
+          <a:ext cx="4358880" cy="3214800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -595,7 +595,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.29"/>
@@ -647,6 +647,9 @@
       <c r="G2" s="1" t="n">
         <v>0.6</v>
       </c>
+      <c r="I2" s="0" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -670,6 +673,9 @@
       <c r="G3" s="1" t="n">
         <v>1.4</v>
       </c>
+      <c r="I3" s="0" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
@@ -698,6 +704,9 @@
       <c r="G5" s="1" t="n">
         <v>60</v>
       </c>
+      <c r="I5" s="0" t="n">
+        <v>102400</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -812,6 +821,9 @@
       </c>
       <c r="G10" s="1" t="n">
         <v>16</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <v>8192</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>